<commit_message>
BOM-Import: Bilder je BOM hochladen (Dateiname = BOM-ID)
Upload zu ImgBB als gemeinsame Funktion uploadToImgbb; schlägt ein Bild
fehl, wird nichts gespeichert. Anleitung in der Vorlage ergänzt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Produktions_BOM_App/BOM-Vorlage.xlsx
+++ b/Produktions_BOM_App/BOM-Vorlage.xlsx
@@ -5609,7 +5609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I25"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5623,6 +5623,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="6" t="inlineStr">
         <is>
@@ -5630,6 +5631,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="7" t="inlineStr">
         <is>
@@ -5675,7 +5677,7 @@
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>5.  Vorschau prüfen (neu / überschreibt bestehende BOM / Fehler) und „Speichern“ klicken.</t>
+          <t>5.  Vorschau prüfen (neu / überschreibt / Fehler), optional „📷 Bilder hinzufügen“ (Dateiname = BOM-ID, z. B. 49284241.jpg), dann „Speichern“ klicken.</t>
         </is>
       </c>
     </row>
@@ -5717,6 +5719,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>

</xml_diff>